<commit_message>
Update daily BIST tracking Excel
</commit_message>
<xml_diff>
--- a/Yüzde.xlsx
+++ b/Yüzde.xlsx
@@ -442,7 +442,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>11.09.2026 20:53:48</t>
+          <t>14.09.2026 20:53:52</t>
         </is>
       </c>
     </row>
@@ -477,7 +477,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -497,7 +497,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -1044,26 +1044,26 @@
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="n">
-        <v>436</v>
+        <v>426</v>
       </c>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="n">
-        <v>0.23</v>
+        <v>-2.07</v>
       </c>
       <c r="O6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P6" t="n">
         <v>440.75</v>
       </c>
       <c r="Q6" t="n">
-        <v>432</v>
+        <v>426</v>
       </c>
       <c r="R6" t="n">
         <v>1.32</v>
       </c>
       <c r="S6" t="n">
-        <v>-0.6899999999999999</v>
+        <v>-2.07</v>
       </c>
       <c r="T6" t="n">
         <v>14505.48</v>
@@ -1117,26 +1117,26 @@
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="n">
-        <v>20</v>
+        <v>19.7</v>
       </c>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="n">
-        <v>0</v>
+        <v>-1.5</v>
       </c>
       <c r="O7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P7" t="n">
         <v>20</v>
       </c>
       <c r="Q7" t="n">
-        <v>20</v>
+        <v>19.52</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>0</v>
+        <v>-2.4</v>
       </c>
       <c r="T7" t="n">
         <v>14467.25</v>

</xml_diff>